<commit_message>
test(mock-data): add SQL example fixtures and update QA checklist
</commit_message>
<xml_diff>
--- a/mock-data/术语配置导入.xlsx
+++ b/mock-data/术语配置导入.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -588,7 +588,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>毕业生初次就业的月平均起薪，单位元/月，对应“就业质量”表“平均起薪(元/月)”字段。</t>
+          <t>毕业生初次就业的月平均起薪，单位元/月，对应“就业质量”表“平均起薪(元/月)”字段。单专业直接取字段；跨专业、院系或全校汇总时必须按毕业生数加权：Σ(平均起薪×毕业生数)÷Σ毕业生数，不得对专业起薪取简单平均。</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>支出合计(万元)×10000÷在校生数(人)，单位元；相关数据见“财务收支”和“办学条件”表。</t>
+          <t>单位元，直接取“财务收支”表的“生均教育经费(元)”字段；不要用支出合计或在读学生数重新计算。</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1106,6 +1106,34 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>课程教学</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>课程成绩,课程</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>对应“课程教学”表，按学年×学期×院系×专业×课程记录，同名课程可能跨学期存在。查询课程成绩或及格率时，必须同时输出学年、学期和院系名称以唯一定位；平均成绩与及格率是两个独立字段。</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>本地mock数据</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>